<commit_message>
Simplify sheet: drop tune/key/author/composer, adopt sadr/ajz/yatim terms
</commit_message>
<xml_diff>
--- a/content/Template.xlsx
+++ b/content/Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="36">
   <si>
     <t>رقم الترنيمة</t>
   </si>
@@ -23,21 +23,9 @@
     <t>العنوان</t>
   </si>
   <si>
-    <t>نظم</t>
-  </si>
-  <si>
     <t>مقياس الكلام</t>
   </si>
   <si>
-    <t>كورد</t>
-  </si>
-  <si>
-    <t>المؤلف</t>
-  </si>
-  <si>
-    <t>الملحن</t>
-  </si>
-  <si>
     <t>القرار</t>
   </si>
   <si>
@@ -47,10 +35,10 @@
     <t>رقم البيت</t>
   </si>
   <si>
-    <t>الشطر الأول</t>
-  </si>
-  <si>
-    <t>الشطر الثاني</t>
+    <t>الصَّدْر</t>
+  </si>
+  <si>
+    <t>العَجُز</t>
   </si>
   <si>
     <t>ملاحظات</t>
@@ -62,21 +50,9 @@
     <t>أنت تعرفني</t>
   </si>
   <si>
-    <t>DENVER</t>
-  </si>
-  <si>
     <t>8.8.8.8</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>مزمور ١٣٩</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>بيت</t>
   </si>
   <si>
@@ -110,7 +86,7 @@
     <t>وفكِّي</t>
   </si>
   <si>
-    <t>نصفان متجاوران</t>
+    <t>صدر وعجز</t>
   </si>
   <si>
     <t>(٣)</t>
@@ -119,6 +95,9 @@
     <t>أنتَ تعرفُ كلَّ أفكاري</t>
   </si>
   <si>
+    <t>يتيم: صدر فقط</t>
+  </si>
+  <si>
     <t>طُرُقي ليستْ عنكَ خفيَّة</t>
   </si>
   <si>
@@ -128,13 +107,13 @@
     <t>١. كل سطر في الكتاب = صف في الجدول. لا تدمج أسطراً في خلية واحدة.</t>
   </si>
   <si>
-    <t>٢. رقم الترنيمة وعنوانها ومعلوماتها (نظم، مقياس الكلام، كورد، المؤلف، الملحن، القرار) تُكتب في أول صف فقط؛ اتركها فارغة في بقية الصفوف.</t>
+    <t>٢. رقم الترنيمة وعنوانها ومقياس الكلام والقرار تُكتب في أول صف فقط؛ اتركها فارغة في بقية الصفوف.</t>
   </si>
   <si>
     <t>٣. رقم البيت بين قوسين في أول سطر فقط: (١). اتركه فارغاً في تتمة البيت نفسه.</t>
   </si>
   <si>
-    <t>٤. النصفان المتجاوران: الأول في «الشطر الأول» والثاني في «الشطر الثاني». السطر الكامل: املأ الأول فقط.</t>
+    <t>٤. البيت من شطرين: الصَّدْر في عموده والعَجُز في عموده. واليَتيم (سطر واحد): املأ الصدر فقط.</t>
   </si>
   <si>
     <t>٥. اللازمة (القرار): صف مستقل في موضعه بالكتاب، واختر «لازمة» من قائمة «نوع السطر».</t>
@@ -544,22 +523,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="7" width="18" customWidth="1"/>
-    <col min="8" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="12" width="40" customWidth="1"/>
-    <col min="13" max="13" width="30" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -587,268 +563,184 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+    </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="2" t="s">
+      <c r="H4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" s="2" t="s">
+    </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="H6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="2" t="s">
+    </row>
+    <row r="7" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="نوع السطر" error="اختر «بيت» أو «لازمة» من القائمة" sqref="I2:I2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="نوع السطر" error="اختر «بيت» أو «لازمة» من القائمة" sqref="E2:E2000">
       <formula1>"بيت,لازمة"</formula1>
     </dataValidation>
   </dataValidations>
@@ -867,47 +759,47 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" ht="8" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adopt book terms: maqta/stanza, bayt tam/mashtur; verseOf correction
</commit_message>
<xml_diff>
--- a/content/Template.xlsx
+++ b/content/Template.xlsx
@@ -29,10 +29,10 @@
     <t>القرار</t>
   </si>
   <si>
-    <t>نوع السطر</t>
-  </si>
-  <si>
-    <t>رقم البيت</t>
+    <t>نوع المقطع</t>
+  </si>
+  <si>
+    <t>رقم المقطع</t>
   </si>
   <si>
     <t>الصَّدْر</t>
@@ -53,7 +53,7 @@
     <t>8.8.8.8</t>
   </si>
   <si>
-    <t>بيت</t>
+    <t>مقطع</t>
   </si>
   <si>
     <t>(١)</t>
@@ -68,7 +68,7 @@
     <t>تعرفُ مَضْجَعِي</t>
   </si>
   <si>
-    <t>سطر بلا رقم بيت = تتمة البيت السابق</t>
+    <t>سطر بلا رقم مقطع = تتمة المقطع السابق</t>
   </si>
   <si>
     <t>لازمة</t>
@@ -86,7 +86,7 @@
     <t>وفكِّي</t>
   </si>
   <si>
-    <t>صدر وعجز</t>
+    <t>بيت تام: صدر وعجز</t>
   </si>
   <si>
     <t>(٣)</t>
@@ -95,7 +95,7 @@
     <t>أنتَ تعرفُ كلَّ أفكاري</t>
   </si>
   <si>
-    <t>يتيم: صدر فقط</t>
+    <t>مشطور: صدر فقط</t>
   </si>
   <si>
     <t>طُرُقي ليستْ عنكَ خفيَّة</t>
@@ -104,19 +104,19 @@
     <t>التعليمات</t>
   </si>
   <si>
-    <t>١. كل سطر في الكتاب = صف في الجدول. لا تدمج أسطراً في خلية واحدة.</t>
+    <t>١. كل بيت في الكتاب = صف في الجدول. لا تدمج أبياتاً في خلية واحدة.</t>
   </si>
   <si>
     <t>٢. رقم الترنيمة وعنوانها ومقياس الكلام والقرار تُكتب في أول صف فقط؛ اتركها فارغة في بقية الصفوف.</t>
   </si>
   <si>
-    <t>٣. رقم البيت بين قوسين في أول سطر فقط: (١). اتركه فارغاً في تتمة البيت نفسه.</t>
-  </si>
-  <si>
-    <t>٤. البيت من شطرين: الصَّدْر في عموده والعَجُز في عموده. واليَتيم (سطر واحد): املأ الصدر فقط.</t>
-  </si>
-  <si>
-    <t>٥. اللازمة (القرار): صف مستقل في موضعه بالكتاب، واختر «لازمة» من قائمة «نوع السطر».</t>
+    <t>٣. رقم المقطع بين قوسين في أول بيت فقط: (١). اتركه فارغاً في تتمة المقطع نفسه.</t>
+  </si>
+  <si>
+    <t>٤. البيت التام: الصَّدْر في عموده والعَجُز في عموده. والمَشْطور (بيت من صدر واحد): املأ الصدر فقط.</t>
+  </si>
+  <si>
+    <t>٥. اللازمة (القرار): صف مستقل في موضعها بالكتاب، واختر «لازمة» من قائمة «نوع المقطع».</t>
   </si>
   <si>
     <t>٦. عمود «ملاحظات» لك وللمحرر فقط — لا يدخل التطبيق أبداً.</t>
@@ -740,8 +740,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="نوع السطر" error="اختر «بيت» أو «لازمة» من القائمة" sqref="E2:E2000">
-      <formula1>"بيت,لازمة"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="نوع المقطع" error="اختر «مقطع» أو «لازمة» من القائمة" sqref="E2:E2000">
+      <formula1>"مقطع,لازمة"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Western digits throughout UI, seed, template and importer labels
</commit_message>
<xml_diff>
--- a/content/Template.xlsx
+++ b/content/Template.xlsx
@@ -44,7 +44,7 @@
     <t>ملاحظات</t>
   </si>
   <si>
-    <t>٧</t>
+    <t>7</t>
   </si>
   <si>
     <t>أنت تعرفني</t>
@@ -56,7 +56,7 @@
     <t>مقطع</t>
   </si>
   <si>
-    <t>(١)</t>
+    <t>(1)</t>
   </si>
   <si>
     <t>أنتَ تعرفُني</t>
@@ -77,7 +77,7 @@
     <t>أنتَ تعرفُني، تعرفُ قلبي</t>
   </si>
   <si>
-    <t>(٢)</t>
+    <t>(2)</t>
   </si>
   <si>
     <t>تعرفُ قِفْلي</t>
@@ -89,7 +89,7 @@
     <t>بيت تام: صدر وعجز</t>
   </si>
   <si>
-    <t>(٣)</t>
+    <t>(3)</t>
   </si>
   <si>
     <t>أنتَ تعرفُ كلَّ أفكاري</t>
@@ -110,7 +110,7 @@
     <t>٢. رقم الترنيمة وعنوانها ومقياس الكلام والقرار تُكتب في أول صف فقط؛ اتركها فارغة في بقية الصفوف.</t>
   </si>
   <si>
-    <t>٣. رقم المقطع بين قوسين في أول بيت فقط: (١). اتركه فارغاً في تتمة المقطع نفسه.</t>
+    <t>٣. رقم المقطع بين قوسين في أول بيت فقط: (1). اتركه فارغاً في تتمة المقطع نفسه.</t>
   </si>
   <si>
     <t>٤. البيت التام: الصَّدْر في عموده والعَجُز في عموده. والمَشْطور (بيت من صدر واحد): املأ الصدر فقط.</t>

</xml_diff>

<commit_message>
Optional per-hymn EN/DE translations: template sheets, importer merge, loader fallback
</commit_message>
<xml_diff>
--- a/content/Template.xlsx
+++ b/content/Template.xlsx
@@ -8,14 +8,16 @@
   </bookViews>
   <sheets>
     <sheet sheetId="1" name="ترانيم" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="تعليمات" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="EN - English" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="DE - Deutsch" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="تعليمات" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="76">
   <si>
     <t>رقم الترنيمة</t>
   </si>
@@ -101,6 +103,123 @@
     <t>طُرُقي ليستْ عنكَ خفيَّة</t>
   </si>
   <si>
+    <t>Hymn No.</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Meter</t>
+  </si>
+  <si>
+    <t>Chorus label</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>Stanza No.</t>
+  </si>
+  <si>
+    <t>First half</t>
+  </si>
+  <si>
+    <t>Second half</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>You Know Me</t>
+  </si>
+  <si>
+    <t>Refrain</t>
+  </si>
+  <si>
+    <t>verse</t>
+  </si>
+  <si>
+    <t>You know me</t>
+  </si>
+  <si>
+    <t>You know my resting place</t>
+  </si>
+  <si>
+    <t>DRAFT — replace with your own wording</t>
+  </si>
+  <si>
+    <t>refrain</t>
+  </si>
+  <si>
+    <t>You know me, You know my heart</t>
+  </si>
+  <si>
+    <t>You know my lock</t>
+  </si>
+  <si>
+    <t>and my key</t>
+  </si>
+  <si>
+    <t>You know all my thoughts</t>
+  </si>
+  <si>
+    <t>My ways are not hidden from You</t>
+  </si>
+  <si>
+    <t>Liednr.</t>
+  </si>
+  <si>
+    <t>Titel</t>
+  </si>
+  <si>
+    <t>Metrum</t>
+  </si>
+  <si>
+    <t>Kehrvers</t>
+  </si>
+  <si>
+    <t>Art</t>
+  </si>
+  <si>
+    <t>Strophennr.</t>
+  </si>
+  <si>
+    <t>Erste Hälfte</t>
+  </si>
+  <si>
+    <t>Zweite Hälfte</t>
+  </si>
+  <si>
+    <t>Notizen</t>
+  </si>
+  <si>
+    <t>Du kennst mich</t>
+  </si>
+  <si>
+    <t>Strophe</t>
+  </si>
+  <si>
+    <t>Du kennst mein Liegen</t>
+  </si>
+  <si>
+    <t>ENTWURF — bitte ersetzen</t>
+  </si>
+  <si>
+    <t>Du kennst mich, Du kennst mein Herz</t>
+  </si>
+  <si>
+    <t>Du kennst mein Schloss</t>
+  </si>
+  <si>
+    <t>und meinen Schlüssel</t>
+  </si>
+  <si>
+    <t>Du kennst all meine Gedanken</t>
+  </si>
+  <si>
+    <t>Meine Wege sind nicht verborgen vor Dir</t>
+  </si>
+  <si>
     <t>التعليمات</t>
   </si>
   <si>
@@ -122,7 +241,10 @@
     <t>٦. عمود «ملاحظات» لك وللمحرر فقط — لا يدخل التطبيق أبداً.</t>
   </si>
   <si>
-    <t>٧. قبل الإرسال: احذف صفوف المثال (٧. أنت تعرفني) واملأ مكانها.</t>
+    <t>٧. قبل الإرسال: احذف صفوف المثال (7. أنت تعرفني) واملأ مكانها.</t>
+  </si>
+  <si>
+    <t>الترجمة (اختياري تماماً): ورقتا EN وDE بنفس الشكل. انسخ رقم الترنيمة نفسه وترجم النص فقط — أي ترنيمة بلا صفوف هناك تظهر بالعربية. ابدأ بترنيمة واحدة متى شئت.</t>
   </si>
 </sst>
 </file>
@@ -173,13 +295,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -751,15 +876,471 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Kind" error="Pick verse or refrain from the list" sqref="E2:E2000">
+      <formula1>"verse,refrain"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Art" error="Strophe oder Kehrvers aus der Liste wählen" sqref="E2:E2000">
+      <formula1>"Strophe,Kehrvers"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>28</v>
+    <row r="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="2" ht="8" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -769,37 +1350,47 @@
     </row>
     <row r="3" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" ht="8" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>